<commit_message>
Prueba QA R5K_v3.pkl v1.0
</commit_message>
<xml_diff>
--- a/output/metricas_por_hoja v0.1.xlsx
+++ b/output/metricas_por_hoja v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae46519d9f6f6d4/2025/Curso Oracle ONE/Hackaton/testing/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E93A5D8-88E1-434F-BA67-36A5A93C6D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{8E93A5D8-88E1-434F-BA67-36A5A93C6D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{570FC2DC-1521-47EF-86CB-3C04159D533C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -441,269 +441,269 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="B2:F16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2">
+      <c r="C3" s="2">
         <v>0.91249999999999998</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D3" s="2">
         <v>0.88372093023255816</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E3" s="2">
         <v>0.95</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F3" s="2">
         <v>0.91566265060240959</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2">
+      <c r="C4" s="2">
         <v>0.91874999999999996</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D4" s="2">
         <v>0.86021505376344087</v>
       </c>
-      <c r="D3" s="2">
-        <v>1</v>
-      </c>
-      <c r="E3" s="2">
+      <c r="E4" s="2">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2">
         <v>0.92485549132947975</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="2">
+      <c r="C5" s="2">
         <v>0.88749999999999996</v>
       </c>
-      <c r="C4" s="2">
+      <c r="D5" s="2">
         <v>0.82978723404255317</v>
       </c>
-      <c r="D4" s="2">
+      <c r="E5" s="2">
         <v>0.97499999999999998</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F5" s="2">
         <v>0.89655172413793105</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2">
+      <c r="C6" s="2">
         <v>0.80625000000000002</v>
       </c>
-      <c r="C5" s="2">
+      <c r="D6" s="2">
         <v>0.7289719626168224</v>
       </c>
-      <c r="D5" s="2">
+      <c r="E6" s="2">
         <v>0.97499999999999998</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F6" s="2">
         <v>0.83422459893048129</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="2">
+      <c r="C7" s="2">
         <v>0.8125</v>
       </c>
-      <c r="C6" s="2">
+      <c r="D7" s="2">
         <v>0.73148148148148151</v>
       </c>
-      <c r="D6" s="2">
+      <c r="E7" s="2">
         <v>0.98750000000000004</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F7" s="2">
         <v>0.84042553191489366</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2">
+      <c r="C8" s="2">
         <v>0.81874999999999998</v>
       </c>
-      <c r="C7" s="2">
+      <c r="D8" s="2">
         <v>0.73394495412844041</v>
       </c>
-      <c r="D7" s="2">
-        <v>1</v>
-      </c>
-      <c r="E7" s="2">
+      <c r="E8" s="2">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2">
         <v>0.84656084656084651</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="2">
-        <v>1</v>
-      </c>
-      <c r="C8" s="2">
-        <v>1</v>
-      </c>
-      <c r="D8" s="2">
-        <v>1</v>
-      </c>
-      <c r="E8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C9" s="2">
+        <v>1</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2">
+      <c r="C10" s="2">
         <v>0.76</v>
       </c>
-      <c r="C9" s="2">
-        <v>1</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="D10" s="2">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2">
         <v>0.76</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F10" s="2">
         <v>0.86363636363636365</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="2">
+      <c r="C11" s="2">
         <v>0.79</v>
       </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-      <c r="D10" s="2">
-        <v>0</v>
-      </c>
-      <c r="E10" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="2">
+      <c r="C12" s="2">
         <v>0.92</v>
       </c>
-      <c r="C11" s="2">
-        <v>0</v>
-      </c>
-      <c r="D11" s="2">
-        <v>0</v>
-      </c>
-      <c r="E11" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="2">
+      <c r="C13" s="2">
         <v>0.24</v>
       </c>
-      <c r="C12" s="2">
-        <v>0</v>
-      </c>
-      <c r="D12" s="2">
-        <v>0</v>
-      </c>
-      <c r="E12" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="2">
+      <c r="C14" s="2">
         <v>0.62</v>
       </c>
-      <c r="C13" s="2">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2">
+      <c r="D14" s="2">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2">
         <v>0.62</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F14" s="2">
         <v>0.76543209876543206</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="2">
+      <c r="C15" s="2">
         <v>0.13</v>
       </c>
-      <c r="C14" s="2">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
-      <c r="E14" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
         <v>18</v>
       </c>
-      <c r="B15" s="2">
+      <c r="C16" s="2">
         <v>0.34</v>
       </c>
-      <c r="C15" s="2">
-        <v>1</v>
-      </c>
-      <c r="D15" s="2">
+      <c r="D16" s="2">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2">
         <v>0.34</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F16" s="2">
         <v>0.5074626865671642</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B15">
+  <conditionalFormatting sqref="C3:C16">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -715,7 +715,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C15">
+  <conditionalFormatting sqref="D3:D16">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -727,7 +727,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D15">
+  <conditionalFormatting sqref="E3:E16">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -739,7 +739,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E15">
+  <conditionalFormatting sqref="F3:F16">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>